<commit_message>
OO-9438: update Excel file to import users
</commit_message>
<xml_diff>
--- a/src/test/java/org/olat/modules/curriculum/ui/importwizard/products-finish-test.xlsx
+++ b/src/test/java/org/olat/modules/curriculum/ui/importwizard/products-finish-test.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/srosse/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8D4E7C9-2CB2-6847-9F92-3D982CD05B1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3C0777D-06CE-4C45-B15B-6001494E1713}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2220" yWindow="7240" windowWidth="44600" windowHeight="19180" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="78">
   <si>
     <t>Title *</t>
   </si>
@@ -280,6 +280,9 @@
       </rPr>
       <t>-MODULE-IMPORT-TEST</t>
     </r>
+  </si>
+  <si>
+    <t>Expiration date</t>
   </si>
 </sst>
 </file>
@@ -1390,7 +1393,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.5" bestFit="1" customWidth="1"/>
@@ -1398,10 +1401,11 @@
     <col min="3" max="3" width="11.33203125" bestFit="1"/>
     <col min="4" max="4" width="29.5" bestFit="1"/>
     <col min="5" max="5" width="14.33203125" bestFit="1"/>
-    <col min="6" max="6" width="18.1640625" bestFit="1"/>
+    <col min="6" max="6" width="18.83203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="35.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>38</v>
       </c>
@@ -1418,10 +1422,13 @@
         <v>46</v>
       </c>
       <c r="F1" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>68</v>
       </c>
@@ -1438,10 +1445,13 @@
         <v>7</v>
       </c>
       <c r="F2" s="11">
+        <v>47860.63958333333</v>
+      </c>
+      <c r="G2" s="11">
         <v>46034.63958333333</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>71</v>
       </c>
@@ -1457,7 +1467,7 @@
       <c r="E3" t="s">
         <v>7</v>
       </c>
-      <c r="F3" s="11">
+      <c r="G3" s="11">
         <v>46035.63958333333</v>
       </c>
     </row>

</xml_diff>